<commit_message>
Updated Walter Feels project to version 2.6
</commit_message>
<xml_diff>
--- a/walter-feels/production/walter-feels-bom.xlsx
+++ b/walter-feels/production/walter-feels-bom.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="375" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="386" uniqueCount="251">
   <si>
     <t xml:space="preserve">Designator</t>
   </si>
@@ -123,7 +123,7 @@
     <t xml:space="preserve">1206</t>
   </si>
   <si>
-    <t xml:space="preserve">C6</t>
+    <t xml:space="preserve">C6, C34, C35</t>
   </si>
   <si>
     <t xml:space="preserve">10nF</t>
@@ -186,7 +186,7 @@
     <t xml:space="preserve">2.2μF ±10%, 16V, X5R, 0603 MLCC</t>
   </si>
   <si>
-    <t xml:space="preserve">C19, C23, C25, C27, C29, C59</t>
+    <t xml:space="preserve">C19, C23, C25, C27, C29, C59, C77</t>
   </si>
   <si>
     <t xml:space="preserve">1μF</t>
@@ -248,7 +248,7 @@
     <t xml:space="preserve">33nF ±10%, 50V, X7R, 0603 MLCC</t>
   </si>
   <si>
-    <t xml:space="preserve">C60, C77</t>
+    <t xml:space="preserve">C60</t>
   </si>
   <si>
     <t xml:space="preserve">4.7μF</t>
@@ -319,12 +319,6 @@
     <t xml:space="preserve">18pF ±5%, 50V, C0G, 0603 MLCC</t>
   </si>
   <si>
-    <t xml:space="preserve">C84</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10µF ±10%, 10V, X5R, 0603 MLCC</t>
-  </si>
-  <si>
     <t xml:space="preserve">D1</t>
   </si>
   <si>
@@ -370,7 +364,34 @@
     <t xml:space="preserve">ESDCAN01-2BLY</t>
   </si>
   <si>
-    <t xml:space="preserve">F1</t>
+    <t xml:space="preserve">D4, D5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.2V</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.2V, 0.2W, Zener diode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SOD-523</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MM5Z8V2T1G</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TVS Diode array</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10-UFDFN</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D3V3X4U10LP-7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">F1, F2</t>
   </si>
   <si>
     <t xml:space="preserve">5A Slow</t>
@@ -667,6 +688,21 @@
     <t xml:space="preserve">SI7611DN-T1-GE3</t>
   </si>
   <si>
+    <t xml:space="preserve">Q4, Q6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30V, 25A, 15.1mΩ, N-channel MOSFET</t>
+  </si>
+  <si>
+    <t xml:space="preserve">6-WSON</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Texas Instruments</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CSD17318Q2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Q5</t>
   </si>
   <si>
@@ -697,7 +733,7 @@
     <t xml:space="preserve">64.9kΩ ±1%, 100mW, 50V, 0603 resistor</t>
   </si>
   <si>
-    <t xml:space="preserve">R4, R5, R8, R11</t>
+    <t xml:space="preserve">R4, R5, R8, R11, R26, R29, R30, R31, R32, R33</t>
   </si>
   <si>
     <t xml:space="preserve">10kΩ</t>
@@ -827,6 +863,15 @@
     <t xml:space="preserve">KRL3216T4-M-R004-F-T1</t>
   </si>
   <si>
+    <t xml:space="preserve">R16, R17, R18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.2MΩ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.2MΩ ±1%, 100mW, 50V, 0603 resistor</t>
+  </si>
+  <si>
     <t xml:space="preserve">R19, R21</t>
   </si>
   <si>
@@ -899,9 +944,6 @@
     <t xml:space="preserve">TSSOP-16</t>
   </si>
   <si>
-    <t xml:space="preserve">Texas Instruments</t>
-  </si>
-  <si>
     <t xml:space="preserve">MAX3221IPWR</t>
   </si>
   <si>
@@ -999,18 +1041,6 @@
   </si>
   <si>
     <t xml:space="preserve">MAX17291ATA+T</t>
-  </si>
-  <si>
-    <t xml:space="preserve">U13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SD-card EMI filter with built-in termination resistors</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DFN-16</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CM1624-08DE</t>
   </si>
   <si>
     <t xml:space="preserve">U14</t>
@@ -1086,7 +1116,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -1099,6 +1129,13 @@
       <right style="hair"/>
       <top style="hair"/>
       <bottom style="hair"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
@@ -1127,7 +1164,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1149,6 +1186,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1343,8 +1388,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G67"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:G73"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="56.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.11"/>
@@ -1354,7 +1399,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="19.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="23.66"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1020" min="8" style="1" width="11.52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16380" style="1" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16382" min="16380" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16383" style="1" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1486,7 +1532,7 @@
         <v>14</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F6" s="4" t="s">
         <v>10</v>
@@ -1647,7 +1693,7 @@
         <v>14</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>10</v>
@@ -1821,231 +1867,231 @@
       <c r="A21" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B21" s="5" t="s">
-        <v>19</v>
-      </c>
+      <c r="B21" s="5"/>
       <c r="C21" s="5" t="s">
         <v>71</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>14</v>
+        <v>72</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>10</v>
+        <v>74</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="B22" s="5"/>
+        <v>75</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>76</v>
+      </c>
       <c r="C22" s="5" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
       <c r="E22" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>77</v>
-      </c>
-      <c r="B23" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B23" s="5"/>
+      <c r="C23" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="D23" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="E23" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="G23" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>88</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="F24" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E23" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F23" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G23" s="5" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B24" s="5"/>
-      <c r="C24" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>80</v>
-      </c>
-      <c r="E24" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>86</v>
+      <c r="G24" s="7" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="E25" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F25" s="4" t="s">
+      <c r="A25" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="G25" s="5" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="6" t="s">
         <v>91</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>92</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="G25" s="7" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="B26" s="5"/>
+        <v>94</v>
+      </c>
+      <c r="B26" s="5" t="s">
+        <v>95</v>
+      </c>
       <c r="C26" s="5" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>94</v>
+        <v>21</v>
       </c>
       <c r="E26" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B27" s="5"/>
       <c r="C27" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="G27" s="5" t="n">
-        <v>693072010801</v>
+        <v>102</v>
+      </c>
+      <c r="G27" s="5" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B28" s="6"/>
+        <v>104</v>
+      </c>
+      <c r="B28" s="5"/>
       <c r="C28" s="5" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="E28" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G28" s="5" t="n">
-        <v>1071010</v>
+        <v>693072010801</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>105</v>
-      </c>
-      <c r="B29" s="6"/>
+        <v>108</v>
+      </c>
+      <c r="B29" s="8"/>
       <c r="C29" s="5" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="G29" s="5" t="n">
-        <v>1990070</v>
+        <v>1071010</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>107</v>
-      </c>
-      <c r="B30" s="5"/>
+        <v>112</v>
+      </c>
+      <c r="B30" s="8"/>
       <c r="C30" s="5" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="E30" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="5" t="s">
-        <v>10</v>
+        <v>111</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>1990070</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="B31" s="4"/>
-      <c r="C31" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="B31" s="5"/>
+      <c r="C31" s="5" t="s">
+        <v>115</v>
+      </c>
+      <c r="D31" s="5" t="s">
         <v>110</v>
       </c>
-      <c r="D31" s="5" t="s">
-        <v>103</v>
-      </c>
       <c r="E31" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F31" s="4" t="s">
         <v>10</v>
@@ -2056,143 +2102,143 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>111</v>
-      </c>
-      <c r="B32" s="5" t="s">
-        <v>112</v>
-      </c>
-      <c r="C32" s="5" t="s">
-        <v>113</v>
+        <v>116</v>
+      </c>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4" t="s">
+        <v>117</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>99</v>
+        <v>110</v>
       </c>
       <c r="E32" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>114</v>
+        <v>10</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>115</v>
+        <v>10</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>116</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
+      </c>
+      <c r="B33" s="5" t="s">
+        <v>119</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="E33" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="B34" s="6" t="s">
-        <v>112</v>
+        <v>123</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>124</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="E34" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>114</v>
+        <v>126</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="B35" s="7"/>
+        <v>128</v>
+      </c>
+      <c r="B35" s="8" t="s">
+        <v>119</v>
+      </c>
       <c r="C35" s="5" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="E35" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="B36" s="5"/>
+        <v>131</v>
+      </c>
+      <c r="B36" s="9"/>
       <c r="C36" s="5" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>130</v>
+        <v>106</v>
       </c>
       <c r="E36" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>81</v>
+        <v>133</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B37" s="5"/>
       <c r="C37" s="5" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="B38" s="5"/>
       <c r="C38" s="5" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>137</v>
@@ -2201,94 +2247,90 @@
         <v>1</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>138</v>
+        <v>79</v>
       </c>
       <c r="G38" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B39" s="5"/>
       <c r="C39" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="E39" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>75</v>
+        <v>145</v>
       </c>
       <c r="G39" s="5" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>144</v>
-      </c>
-      <c r="B40" s="5" t="s">
-        <v>145</v>
-      </c>
+        <v>147</v>
+      </c>
+      <c r="B40" s="5"/>
       <c r="C40" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="D40" s="5" t="s">
-        <v>14</v>
+        <v>149</v>
       </c>
       <c r="E40" s="4" t="n">
         <v>2</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G40" s="5" t="s">
-        <v>10</v>
+        <v>151</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="B41" s="5" t="s">
-        <v>148</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="B41" s="5"/>
       <c r="C41" s="5" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="D41" s="5" t="s">
-        <v>14</v>
+        <v>154</v>
       </c>
       <c r="E41" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>10</v>
+        <v>73</v>
       </c>
       <c r="G41" s="5" t="s">
-        <v>10</v>
+        <v>155</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="B42" s="5" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E42" s="4" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F42" s="4" t="s">
         <v>10</v>
@@ -2299,19 +2341,19 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="B43" s="5" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="C43" s="5" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E43" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F43" s="4" t="s">
         <v>10</v>
@@ -2322,19 +2364,19 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="B44" s="5" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="C44" s="5" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E44" s="4" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F44" s="4" t="s">
         <v>10</v>
@@ -2345,19 +2387,19 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B45" s="5" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="C45" s="5" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E45" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F45" s="4" t="s">
         <v>10</v>
@@ -2368,13 +2410,13 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="4" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="B46" s="5" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="C46" s="5" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>14</v>
@@ -2391,19 +2433,19 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="B47" s="5" t="s">
-        <v>151</v>
+        <v>172</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E47" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>10</v>
@@ -2414,111 +2456,111 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B48" s="5" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C48" s="5" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="D48" s="5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E48" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>170</v>
+        <v>10</v>
       </c>
       <c r="G48" s="5" t="s">
-        <v>171</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B49" s="5" t="s">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="E49" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>170</v>
+        <v>10</v>
       </c>
       <c r="G49" s="5" t="s">
-        <v>175</v>
+        <v>10</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="B50" s="5" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E50" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>10</v>
+        <v>182</v>
       </c>
       <c r="G50" s="5" t="s">
-        <v>10</v>
+        <v>183</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B51" s="5" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="C51" s="5" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="E51" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>10</v>
+        <v>182</v>
       </c>
       <c r="G51" s="5" t="s">
-        <v>10</v>
+        <v>187</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="B52" s="5" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="C52" s="5" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E52" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>10</v>
@@ -2529,19 +2571,19 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="B53" s="5" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="C53" s="5" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>14</v>
       </c>
       <c r="E53" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F53" s="4" t="s">
         <v>10</v>
@@ -2552,13 +2594,13 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="B54" s="5" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="C54" s="5" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>14</v>
@@ -2575,13 +2617,13 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="B55" s="5" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="C55" s="5" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>14</v>
@@ -2598,13 +2640,13 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B56" s="5" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="C56" s="5" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>14</v>
@@ -2621,235 +2663,286 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>197</v>
-      </c>
-      <c r="B57" s="5"/>
+        <v>203</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>204</v>
+      </c>
       <c r="C57" s="5" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="D57" s="5" t="s">
-        <v>199</v>
+        <v>14</v>
       </c>
       <c r="E57" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="G57" s="5" t="s">
-        <v>201</v>
+        <v>10</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>202</v>
-      </c>
-      <c r="B58" s="6"/>
+        <v>206</v>
+      </c>
+      <c r="B58" s="5" t="s">
+        <v>207</v>
+      </c>
       <c r="C58" s="5" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="D58" s="5" t="s">
-        <v>204</v>
+        <v>14</v>
       </c>
       <c r="E58" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>205</v>
+        <v>10</v>
       </c>
       <c r="G58" s="5" t="s">
-        <v>206</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>207</v>
-      </c>
-      <c r="B59" s="6"/>
+        <v>209</v>
+      </c>
+      <c r="B59" s="5" t="s">
+        <v>210</v>
+      </c>
       <c r="C59" s="5" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>209</v>
+        <v>14</v>
       </c>
       <c r="E59" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="G59" s="5" t="s">
-        <v>210</v>
+        <v>10</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B60" s="6"/>
+        <v>212</v>
+      </c>
+      <c r="B60" s="5"/>
       <c r="C60" s="5" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>204</v>
+        <v>214</v>
       </c>
       <c r="E60" s="4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>200</v>
+        <v>150</v>
       </c>
       <c r="G60" s="5" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B61" s="6"/>
+        <v>216</v>
+      </c>
+      <c r="B61" s="8"/>
       <c r="C61" s="5" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D61" s="5" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E61" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="G61" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="B62" s="6"/>
+        <v>221</v>
+      </c>
+      <c r="B62" s="8"/>
       <c r="C62" s="5" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="D62" s="5" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="E62" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>85</v>
+        <v>150</v>
       </c>
       <c r="G62" s="5" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>222</v>
-      </c>
-      <c r="B63" s="6"/>
+        <v>225</v>
+      </c>
+      <c r="B63" s="8"/>
       <c r="C63" s="5" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="D63" s="5" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="E63" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>85</v>
+        <v>150</v>
       </c>
       <c r="G63" s="5" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>226</v>
-      </c>
-      <c r="B64" s="6"/>
+        <v>228</v>
+      </c>
+      <c r="B64" s="8"/>
       <c r="C64" s="5" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E64" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>95</v>
+        <v>150</v>
       </c>
       <c r="G64" s="5" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>230</v>
-      </c>
-      <c r="B65" s="6"/>
+        <v>232</v>
+      </c>
+      <c r="B65" s="8"/>
       <c r="C65" s="5" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="E65" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>95</v>
+        <v>83</v>
       </c>
       <c r="G65" s="5" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="B66" s="6"/>
+        <v>236</v>
+      </c>
+      <c r="B66" s="8"/>
       <c r="C66" s="5" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="D66" s="5" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="E66" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="G66" s="5" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="B67" s="6"/>
+        <v>240</v>
+      </c>
+      <c r="B67" s="8"/>
       <c r="C67" s="5" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="D67" s="5" t="s">
-        <v>209</v>
+        <v>242</v>
       </c>
       <c r="E67" s="4" t="n">
         <v>1</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>200</v>
+        <v>102</v>
       </c>
       <c r="G67" s="5" t="s">
-        <v>240</v>
-      </c>
-    </row>
+        <v>243</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A68" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B68" s="8"/>
+      <c r="C68" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="D68" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F68" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="G68" s="5" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A69" s="4" t="s">
+        <v>248</v>
+      </c>
+      <c r="B69" s="8"/>
+      <c r="C69" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="E69" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="4" t="s">
+        <v>150</v>
+      </c>
+      <c r="G69" s="5" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="73" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>

</xml_diff>